<commit_message>
Synchronize all four Excel engineering sheets after bidirectional question backfill
</commit_message>
<xml_diff>
--- a/papers/P001/P001_工程复现问题清单_v1.xlsx
+++ b/papers/P001/P001_工程复现问题清单_v1.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Aptos"/>
@@ -19,12 +19,6 @@
       <sz val="11"/>
       <name val="Aptos"/>
       <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Aptos"/>
-      <u/>
-      <color rgb="FF0563C1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -42,7 +36,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF0F5FA"/>
+        <fgColor rgb="FFF1F5F9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -59,18 +53,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -81,15 +72,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="25"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="54" customWidth="1"/>
-    <col min="3" max="3" width="95" customWidth="1"/>
+    <col min="3" max="3" width="103" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="38" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">主题</t>
@@ -106,7 +97,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="92" customHeight="1">
+    <row r="2" ht="93" customHeight="1">
       <c r="A2" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">研究假设（Idea）来源</t>
@@ -126,191 +117,225 @@
     <row r="3" ht="93" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">经典结构先验</t>
+          <t xml:space="preserve">市场上下文</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">WorldQuant 101 Alpha到底是什么、来自哪里？</t>
+          <t xml:space="preserve">它是否像P005一样每天生成市场环境描述交给LLM？</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">源于WorldQuant《101 Formulaic Alphas》；作者放在101_alpha.json，含因子ID、输入字段和Python表达式。它是供Writer参考的经典公式示例，并非强制语法约束。</t>
+          <t xml:space="preserve">Writer主要接受自然语言研究假设、两个知识库的检索结果及反馈，未见独立的“每日行情统计→市场自然语言摘要”模块。OHLCV主要进入因子计算和回测，不能把行情表等同于直接输入Writer的市场描述。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="93" customHeight="1">
       <c r="A4" t="inlineStr" s="0">
         <is>
+          <t xml:space="preserve">经典结构先验</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">WorldQuant 101 Alpha到底是什么、来自哪里？</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">源于WorldQuant《101 Formulaic Alphas》；作者放在101_alpha.json，含因子ID、输入字段和Python表达式。它是供Writer参考的经典公式示例，并非强制语法约束。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="83" customHeight="1">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">两个知识库</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="0">
+      <c r="B5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">101 KB与Main KB各存什么，为什么分开？</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="0">
+      <c r="C5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">101 KB是已有经典公式；Main KB保存之前筛选出的因子、想法、代码和IC/Sharpe等表现，供之后复用。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="93" customHeight="1">
-      <c r="A5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">检索方法</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">是LLM阅读整个KB，还是程序预选参考？</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Python先用all-MiniLM-L6-v2 Embedding检索；101 KB取最相似1条，Main KB用0.7×语义相似度+0.3×(IC+1)排序后取1条。LLM没有直接遍历整个KB。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="93" customHeight="1">
       <c r="A6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Writer输入</t>
+          <t xml:space="preserve">检索方法</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Idea、两种先验和反馈究竟怎样输入？</t>
+          <t xml:space="preserve">是LLM阅读整个KB，还是程序预选参考？</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">程序把四部分填进YAML里的user_template，拼成普通文本User Prompt，连同System Prompt、近期对话消息发给LLM；不是四份原始JSON分别供LLM自主检索。</t>
+          <t xml:space="preserve">Python先用all-MiniLM-L6-v2 Embedding检索；101 KB取最相似1条，Main KB用0.7×语义相似度+0.3×(IC+1)排序后取1条。LLM没有直接遍历整个KB。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="93" customHeight="1">
       <c r="A7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">生成结果</t>
+          <t xml:space="preserve">Writer输入</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Writer生成什么、怎样运行？</t>
+          <t xml:space="preserve">Idea、两种先验和反馈究竟怎样输入？</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">生成LaTeX公式及Python因子代码，代码需符合AlphaBase子类的calc(data)接口：用OHLCV DataFrame计算并返回逐日×股票的因子信号。</t>
+          <t xml:space="preserve">程序把四部分填进YAML里的user_template，拼成普通文本User Prompt，连同System Prompt、近期对话消息发给LLM；不是四份原始JSON分别供LLM自主检索。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="93" customHeight="1">
       <c r="A8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">内循环</t>
+          <t xml:space="preserve">生成结果</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Judge检查什么、如何让Writer修改？</t>
+          <t xml:space="preserve">Writer生成什么、怎样运行？</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">先验Python语法，再由Judge按研究假设一致性、未来信息风险、代码和信号质量评分；未过阈值就把Judge的文字反馈与当轮旧代码再次放进Prompt，通常最多循环若干轮。</t>
+          <t xml:space="preserve">生成LaTeX公式及Python因子代码，代码需符合AlphaBase子类的calc(data)接口：用OHLCV DataFrame计算并返回逐日×股票的因子信号。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="93" customHeight="1">
       <c r="A9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">外循环</t>
+          <t xml:space="preserve">内循环</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reviewer反馈如何传递？会拿上一版代码修改吗？</t>
+          <t xml:space="preserve">Judge检查什么、如何让Writer修改？</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">运行因子并计算IC等指标后，Reviewer给自然语言修改建议，再送进下一轮Writer；外轮重建ContextBuffer，上一版完整代码并未稳定跨轮传递，实际更接近按建议重新生成。</t>
+          <t xml:space="preserve">先验Python语法，再由Judge按研究假设一致性、未来信息风险、代码和信号质量评分；未过阈值就把Judge的文字反馈与当轮旧代码再次放进Prompt，通常最多循环若干轮。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="93" customHeight="1">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">经验写回</t>
+          <t xml:space="preserve">外循环</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">KBUpdater究竟如何把新因子放回知识库？</t>
+          <t xml:space="preserve">Reviewer反馈如何传递？会拿上一版代码修改吗？</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">虽然有KBUpdater类，但实际OuterLoop主要直接保留IC最优候选；IC≥0.01且允许写入时加入Main KB，验证/测试可冻结写入。不是LLM权重训练。</t>
+          <t xml:space="preserve">运行因子并计算IC等指标后，Reviewer给自然语言修改建议，再送进下一轮Writer；外轮重建ContextBuffer，上一版完整代码并未稳定跨轮传递，实际更接近按建议重新生成。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="93" customHeight="1">
       <c r="A11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">自迭代含义</t>
+          <t xml:space="preserve">经验写回</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Self-improving到底改进了什么？</t>
+          <t xml:space="preserve">KBUpdater究竟如何把新因子放回知识库？</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">短期改变候选因子代码（内外循环），长期积累通过筛选的因子样例（Main KB）；没有显示通过SFT/RL更新基础LLM参数。</t>
+          <t xml:space="preserve">虽然有KBUpdater类，但实际OuterLoop主要直接保留IC最优候选；IC≥0.01且允许写入时加入Main KB，验证/测试可冻结写入。不是LLM权重训练。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="93" customHeight="1">
       <c r="A12" t="inlineStr" s="0">
         <is>
+          <t xml:space="preserve">筛选粒度与池级边际</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">根据单因子分数入库，还是看新增因子对整池的边际提升？</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">OuterLoop在候选中取IC最优者，满足IC≥0.01且允许写入才保存到Main KB；没有像P005那样重算加权组合池分数Γ(P)以及新增候选的ΔΓ。历史案例知识库不等于按池级边际维护的组合池。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="83" customHeight="1">
+      <c r="A13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">自迭代含义</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Self-improving到底改进了什么？</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">短期改变候选因子代码（内外循环），长期积累通过筛选的因子样例（Main KB）；没有显示通过SFT/RL更新基础LLM参数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="93" customHeight="1">
+      <c r="A14" t="inlineStr" s="0">
+        <is>
           <t xml:space="preserve">LLM底座</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr" s="0">
+      <c r="B14" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">它用的什么大模型？</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr" s="0">
+      <c r="C14" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">作者公开实现中Writer默认Groq提供的Meta Llama 4 Scout（17B/16E Instruct），可传参替换；Judge/Reviewer也通过LLM调用，模型随配置改变。没有证据这是单独微调的金融模型。</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="93" customHeight="1">
-      <c r="A13" t="inlineStr" s="2">
+    <row r="15" ht="93" customHeight="1">
+      <c r="A15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">源码及复现边界</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr" s="2">
+      <c r="B15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">作者代码公开到什么程度？</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr" s="2">
+      <c r="C15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">作者发布Writer/Judge/Reviewer、检索、提示词、循环和API实现，但公开目录缺src/data、知识库默认路径写死作者机器、LLM配置文件名有差异；目前仅源码核查，未实际跑通端到端。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C13"/>
+  <autoFilter ref="A1:C15"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync P006 and retrospective P001–P005 engineering Excel tables with latest CSV
</commit_message>
<xml_diff>
--- a/papers/P001/P001_工程复现问题清单_v1.xlsx
+++ b/papers/P001/P001_工程复现问题清单_v1.xlsx
@@ -36,7 +36,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
+        <fgColor rgb="FFF2F5F9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -55,13 +55,13 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -72,15 +72,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="54" customWidth="1"/>
-    <col min="3" max="3" width="103" customWidth="1"/>
+    <col min="2" max="2" width="53" customWidth="1"/>
+    <col min="3" max="3" width="92" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="38" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">主题</t>
@@ -97,7 +97,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="93" customHeight="1">
+    <row r="2" ht="82" customHeight="1">
       <c r="A2" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">研究假设（Idea）来源</t>
@@ -114,7 +114,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="93" customHeight="1">
+    <row r="3" ht="94" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">市场上下文</t>
@@ -131,7 +131,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="93" customHeight="1">
+    <row r="4" ht="94" customHeight="1">
       <c r="A4" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">经典结构先验</t>
@@ -148,7 +148,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="83" customHeight="1">
+    <row r="5" ht="82" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">两个知识库</t>
@@ -165,7 +165,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="93" customHeight="1">
+    <row r="6" ht="94" customHeight="1">
       <c r="A6" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">检索方法</t>
@@ -182,7 +182,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="93" customHeight="1">
+    <row r="7" ht="94" customHeight="1">
       <c r="A7" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Writer输入</t>
@@ -199,7 +199,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="93" customHeight="1">
+    <row r="8" ht="82" customHeight="1">
       <c r="A8" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">生成结果</t>
@@ -216,7 +216,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="93" customHeight="1">
+    <row r="9" ht="82" customHeight="1">
       <c r="A9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">内循环</t>
@@ -233,7 +233,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="93" customHeight="1">
+    <row r="10" ht="94" customHeight="1">
       <c r="A10" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">外循环</t>
@@ -250,7 +250,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="93" customHeight="1">
+    <row r="11" ht="82" customHeight="1">
       <c r="A11" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">经验写回</t>
@@ -267,7 +267,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="93" customHeight="1">
+    <row r="12" ht="94" customHeight="1">
       <c r="A12" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">筛选粒度与池级边际</t>
@@ -284,7 +284,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="83" customHeight="1">
+    <row r="13" ht="82" customHeight="1">
       <c r="A13" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">自迭代含义</t>
@@ -301,41 +301,58 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="93" customHeight="1">
+    <row r="14" ht="94" customHeight="1">
       <c r="A14" t="inlineStr" s="0">
         <is>
+          <t xml:space="preserve">研究调度与优化对象</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">下一步由Bandit在Factor/Model间选择吗？会让LLM提出预测模型架构吗？</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">没有P006式二臂Bandit或因子—模型交替研发。P001以给定Research Idea为起点，Writer按Prompt生成/改良因子，Judge/Reviewer及程序控制内外循环；股票收益预测与回测提供评价，系统不单独让LLM提出新预测模型架构。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="94" customHeight="1">
+      <c r="A15" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">LLM底座</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr" s="0">
+      <c r="B15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">它用的什么大模型？</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr" s="0">
+      <c r="C15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">作者公开实现中Writer默认Groq提供的Meta Llama 4 Scout（17B/16E Instruct），可传参替换；Judge/Reviewer也通过LLM调用，模型随配置改变。没有证据这是单独微调的金融模型。</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="93" customHeight="1">
-      <c r="A15" t="inlineStr" s="2">
+    <row r="16" ht="94" customHeight="1">
+      <c r="A16" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">源码及复现边界</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr" s="2">
+      <c r="B16" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">作者代码公开到什么程度？</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr" s="2">
+      <c r="C16" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">作者发布Writer/Judge/Reviewer、检索、提示词、循环和API实现，但公开目录缺src/data、知识库默认路径写死作者机器、LLM配置文件名有差异；目前仅源码核查，未实际跑通端到端。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C15"/>
+  <autoFilter ref="A1:C16"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync polished P001–P005 Excel engineering tables with new CSV rows
</commit_message>
<xml_diff>
--- a/papers/P001/P001_工程复现问题清单_v1.xlsx
+++ b/papers/P001/P001_工程复现问题清单_v1.xlsx
@@ -30,7 +30,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF142B46"/>
+        <fgColor rgb="FF172D48"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -72,12 +72,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="25"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="53" customWidth="1"/>
-    <col min="3" max="3" width="92" customWidth="1"/>
+    <col min="3" max="3" width="98" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -97,7 +97,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="82" customHeight="1">
+    <row r="2" ht="78" customHeight="1">
       <c r="A2" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">研究假设（Idea）来源</t>
@@ -114,7 +114,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="94" customHeight="1">
+    <row r="3" ht="78" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">市场上下文</t>
@@ -127,11 +127,11 @@
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Writer主要接受自然语言研究假设、两个知识库的检索结果及反馈，未见独立的“每日行情统计→市场自然语言摘要”模块。OHLCV主要进入因子计算和回测，不能把行情表等同于直接输入Writer的市场描述。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="94" customHeight="1">
+          <t xml:space="preserve">LLM主要接收Idea、知识库检索案例及反馈；OHLCV用于因子计算和评价，没有P005那样单独生成的每日市场文字描述。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="86" customHeight="1">
       <c r="A4" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">经典结构先验</t>
@@ -148,211 +148,177 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="82" customHeight="1">
+    <row r="5" ht="86" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">两个知识库</t>
+          <t xml:space="preserve">两个知识库与检索</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">101 KB与Main KB各存什么，为什么分开？</t>
+          <t xml:space="preserve">101 KB、Main KB存什么？参考案例怎样找到？</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">101 KB是已有经典公式；Main KB保存之前筛选出的因子、想法、代码和IC/Sharpe等表现，供之后复用。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="94" customHeight="1">
+          <t xml:space="preserve">101 KB保存WorldQuant经典公式；Main KB保存已筛因子的想法、代码和表现。程序用all-MiniLM-L6-v2做语义检索：101 KB取最相似1条，Main KB按0.7×相似度+0.3×(IC+1)排序取1条，再交给Writer。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="86" customHeight="1">
       <c r="A6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">检索方法</t>
+          <t xml:space="preserve">Writer输入</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">是LLM阅读整个KB，还是程序预选参考？</t>
+          <t xml:space="preserve">Idea、两种先验和反馈究竟怎样输入？</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Python先用all-MiniLM-L6-v2 Embedding检索；101 KB取最相似1条，Main KB用0.7×语义相似度+0.3×(IC+1)排序后取1条。LLM没有直接遍历整个KB。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="94" customHeight="1">
+          <t xml:space="preserve">程序把四部分填进YAML里的user_template，拼成普通文本User Prompt，连同System Prompt、近期对话消息发给LLM；不是四份原始JSON分别供LLM自主检索。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
       <c r="A7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Writer输入</t>
+          <t xml:space="preserve">生成结果</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Idea、两种先验和反馈究竟怎样输入？</t>
+          <t xml:space="preserve">Writer生成什么、怎样运行？</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">程序把四部分填进YAML里的user_template，拼成普通文本User Prompt，连同System Prompt、近期对话消息发给LLM；不是四份原始JSON分别供LLM自主检索。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="82" customHeight="1">
+          <t xml:space="preserve">生成LaTeX公式及Python因子代码，代码需符合AlphaBase子类的calc(data)接口：用OHLCV DataFrame计算并返回逐日×股票的因子信号。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="78" customHeight="1">
       <c r="A8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">生成结果</t>
+          <t xml:space="preserve">内循环</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Writer生成什么、怎样运行？</t>
+          <t xml:space="preserve">Judge检查什么、如何让Writer修改？</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">生成LaTeX公式及Python因子代码，代码需符合AlphaBase子类的calc(data)接口：用OHLCV DataFrame计算并返回逐日×股票的因子信号。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="82" customHeight="1">
+          <t xml:space="preserve">先查Python语法；Judge再看假设是否对齐、是否疑似使用未来信息及代码/信号质量。不达标就把旧代码与文字意见传给Writer修改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78" customHeight="1">
       <c r="A9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">内循环</t>
+          <t xml:space="preserve">外循环</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Judge检查什么、如何让Writer修改？</t>
+          <t xml:space="preserve">Reviewer反馈如何传递？会拿上一版代码修改吗？</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">先验Python语法，再由Judge按研究假设一致性、未来信息风险、代码和信号质量评分；未过阈值就把Judge的文字反馈与当轮旧代码再次放进Prompt，通常最多循环若干轮。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="94" customHeight="1">
+          <t xml:space="preserve">实测IC等指标后，Reviewer给修改建议，供下一轮Writer重新生成；外循环重置ContextBuffer，旧版完整代码未稳定跨轮携带。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">外循环</t>
+          <t xml:space="preserve">知识库写回与筛选</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Reviewer反馈如何传递？会拿上一版代码修改吗？</t>
+          <t xml:space="preserve">新因子怎样进入Main KB？看单因子还是整池增益？</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">运行因子并计算IC等指标后，Reviewer给自然语言修改建议，再送进下一轮Writer；外轮重建ContextBuffer，上一版完整代码并未稳定跨轮传递，实际更接近按建议重新生成。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="82" customHeight="1">
+          <t xml:space="preserve">OuterLoop保留候选中IC最佳者，IC≥0.01且允许写入时保存到Main KB；验证/测试阶段可冻结写入。虽有KBUpdater类，主流程直接筛选；未用P005式整池增量ΔΓ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="78" customHeight="1">
       <c r="A11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">经验写回</t>
+          <t xml:space="preserve">自迭代含义</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">KBUpdater究竟如何把新因子放回知识库？</t>
+          <t xml:space="preserve">Self-improving到底改进了什么？</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">虽然有KBUpdater类，但实际OuterLoop主要直接保留IC最优候选；IC≥0.01且允许写入时加入Main KB，验证/测试可冻结写入。不是LLM权重训练。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="94" customHeight="1">
+          <t xml:space="preserve">改变的是候选代码、Prompt反馈和Main KB成功案例；未报告对基础LLM做SFT/RL参数训练。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="78" customHeight="1">
       <c r="A12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">筛选粒度与池级边际</t>
+          <t xml:space="preserve">研究调度与优化对象</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">根据单因子分数入库，还是看新增因子对整池的边际提升？</t>
+          <t xml:space="preserve">下一步由Bandit在Factor/Model间选择吗？会让LLM提出预测模型架构吗？</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">OuterLoop在候选中取IC最优者，满足IC≥0.01且允许写入才保存到Main KB；没有像P005那样重算加权组合池分数Γ(P)以及新增候选的ΔΓ。历史案例知识库不等于按池级边际维护的组合池。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="82" customHeight="1">
+          <t xml:space="preserve">系统只改因子，由Writer生成、Judge/Reviewer反馈并循环；没有P006的Factor/Model双臂Bandit，也不自主设计下游模型。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="86" customHeight="1">
       <c r="A13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">自迭代含义</t>
+          <t xml:space="preserve">LLM底座</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Self-improving到底改进了什么？</t>
+          <t xml:space="preserve">它用的什么大模型？</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">短期改变候选因子代码（内外循环），长期积累通过筛选的因子样例（Main KB）；没有显示通过SFT/RL更新基础LLM参数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="94" customHeight="1">
+          <t xml:space="preserve">作者公开实现中Writer默认Groq提供的Meta Llama 4 Scout（17B/16E Instruct），可传参替换；Judge/Reviewer也通过LLM调用，模型随配置改变。没有证据这是单独微调的金融模型。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="86" customHeight="1">
       <c r="A14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">研究调度与优化对象</t>
+          <t xml:space="preserve">源码及复现边界</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">下一步由Bandit在Factor/Model间选择吗？会让LLM提出预测模型架构吗？</t>
+          <t xml:space="preserve">作者代码公开到什么程度？</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">没有P006式二臂Bandit或因子—模型交替研发。P001以给定Research Idea为起点，Writer按Prompt生成/改良因子，Judge/Reviewer及程序控制内外循环；股票收益预测与回测提供评价，系统不单独让LLM提出新预测模型架构。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="94" customHeight="1">
-      <c r="A15" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">LLM底座</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">它用的什么大模型？</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">作者公开实现中Writer默认Groq提供的Meta Llama 4 Scout（17B/16E Instruct），可传参替换；Judge/Reviewer也通过LLM调用，模型随配置改变。没有证据这是单独微调的金融模型。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="94" customHeight="1">
-      <c r="A16" t="inlineStr" s="0">
-        <is>
-          <t xml:space="preserve">源码及复现边界</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr" s="0">
-        <is>
-          <t xml:space="preserve">作者代码公开到什么程度？</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr" s="0">
-        <is>
           <t xml:space="preserve">作者发布Writer/Judge/Reviewer、检索、提示词、循环和API实现，但公开目录缺src/data、知识库默认路径写死作者机器、LLM配置文件名有差异；目前仅源码核查，未实际跑通端到端。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C16"/>
+  <autoFilter ref="A1:C14"/>
 </worksheet>
 </file>
</xml_diff>